<commit_message>
if there is approval mapped go to him else default
</commit_message>
<xml_diff>
--- a/public/templates/internal_upload_template.xlsx
+++ b/public/templates/internal_upload_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\timesheet-app\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2EC4AA3-3184-4F03-A989-A03105AF82E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073E0031-487E-41B7-816F-B51A8DCB8EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{013FBE18-F61B-431E-9C57-53EF7E3B5338}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="27">
   <si>
     <t>Email</t>
   </si>
@@ -66,27 +66,12 @@
     <t>SubTeams</t>
   </si>
   <si>
-    <t>BA</t>
-  </si>
-  <si>
     <t>QA</t>
   </si>
   <si>
     <t>DEV</t>
   </si>
   <si>
-    <t>Bristol Bertha</t>
-  </si>
-  <si>
-    <t>Bbertha@slideinsurance.com</t>
-  </si>
-  <si>
-    <t>rshaikh@slideinsurance.com</t>
-  </si>
-  <si>
-    <t>Rahil Shaikh</t>
-  </si>
-  <si>
     <t>Delivery/Scrum Master</t>
   </si>
   <si>
@@ -127,13 +112,19 @@
   </si>
   <si>
     <t>IT Ops</t>
+  </si>
+  <si>
+    <t>sjoginipalli@slideinsurance.com</t>
+  </si>
+  <si>
+    <t>Shravan Kumar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,6 +146,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -184,11 +181,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -524,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5412F18-43F0-4B39-A3A8-2B1B8B345020}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
@@ -547,38 +545,38 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="A2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-    </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
+      <c r="A4" s="1"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
+      <c r="A5" s="1"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
@@ -596,13 +594,13 @@
       <c r="A10" s="1"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="1"/>
+      <c r="A11" s="2"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
+      <c r="A13" s="1"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
@@ -613,17 +611,7 @@
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="1"/>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{03865FB7-B74E-4234-99FA-EE3ECEFDF54B}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{656875D4-773E-40C4-8E01-2F2BC43F934D}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -668,7 +656,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -676,7 +664,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -684,7 +672,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -692,61 +680,61 @@
         <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>